<commit_message>
Practice templates: remove the classification-marking line
Owner direction, 21 October 2026. "[CLASSIFICATION: when filled in, mark as your security classification
guide and PSO direct]" is gone from every practice template: the docx headers, and row 2 of each workbook
sheet (left empty and shrunk, so formulas keep their rows). The training-sample notice stays. A test keeps
the line from returning.
</commit_message>
<xml_diff>
--- a/public/training/library/training-samples/SBD-Training-Hardware-Software-Lists.xlsx
+++ b/public/training/library/training-samples/SBD-Training-Hardware-Software-Lists.xlsx
@@ -31,7 +31,7 @@
     <t xml:space="preserve">SECURE BY DESIGN TRAINING SAMPLE - NOT AN OFFICIAL FORM. For instruction and practice with fictional data only.</t>
   </si>
   <si>
-    <t xml:space="preserve">[CLASSIFICATION: when filled in, mark this document as your security classification guide and PSO direct]</t>
+    <t/>
   </si>
   <si>
     <t xml:space="preserve">Hardware and software lists - training sample</t>
@@ -765,10 +765,8 @@
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
+    <row r="2" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="4" customHeight="1">
+      <c r="A2" s="2"/>
       <c r="B2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -908,10 +906,8 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
+    <row r="2" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="4" customHeight="1">
+      <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -4400,10 +4396,8 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
+    <row r="2" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="4" customHeight="1">
+      <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>

</xml_diff>